<commit_message>
Adding parallel execution functionality to the execution and fixing some minor issues
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/testdata.xlsx
+++ b/src/test/resources/excel/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2e9f1ff2b390a8ed/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\seleniumTesting\POMTestExecution\src\test\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8AA40D74-FBF8-43C4-BF65-6AB151AFCFD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2FDB5B-7E22-432E-BE8B-E532CC8B22FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="38700" windowHeight="15345" activeTab="4" xr2:uid="{5646E030-7350-4DC6-A18A-3CD70EBE5421}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="38700" windowHeight="15345" activeTab="1" xr2:uid="{5646E030-7350-4DC6-A18A-3CD70EBE5421}"/>
   </bookViews>
   <sheets>
     <sheet name="itemsPresent" sheetId="1" r:id="rId1"/>
@@ -19,21 +19,10 @@
     <sheet name="priceCompare" sheetId="4" r:id="rId4"/>
     <sheet name="requestValidation" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -512,7 +501,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>